<commit_message>
Doral July 2026: set Cash Payments Owed to $224 per office
Office expense lines are now License Rent $500, Systems $224, Cash Payments Owed
$224 (was $589). Net to Doral is $7,086.82. Regenerated both PDFs and the
workbook; gross commission unchanged at $9,462.56.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QzWo6EPP234vFHwQr61xeD
</commit_message>
<xml_diff>
--- a/commissions/2026-07/Doral_Binder_Book_July_2026_Commissions.xlsx
+++ b/commissions/2026-07/Doral_Binder_Book_July_2026_Commissions.xlsx
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>-589</v>
+        <v>-224</v>
       </c>
     </row>
     <row r="20">
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>6721.82</v>
+        <v>7086.82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Doral July 2026: record Ocean Harbor in full, drop Cash Payments line
Record all five Ocean Harbor producer-6883 statement lines as shown, including
Ertas Meral (+$118.91) and Morin George (-$64.87), so the section foots to the
statement's $250.08 Commission Due. Remove the Cash Payments Owed expense line
for now (office lines are License Rent $500 and Systems $224).

Gross commission $9,516.60; net to Doral $7,356.75. Regenerated both PDFs and
the workbook.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QzWo6EPP234vFHwQr61xeD
</commit_message>
<xml_diff>
--- a/commissions/2026-07/Doral_Binder_Book_July_2026_Commissions.xlsx
+++ b/commissions/2026-07/Doral_Binder_Book_July_2026_Commissions.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -597,10 +597,10 @@
         <v>173.16</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>22.88</v>
+        <v>76.92</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>196.04</v>
+        <v>250.08</v>
       </c>
     </row>
     <row r="11">
@@ -613,10 +613,10 @@
         <v>3057.29</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>6405.27</v>
+        <v>6459.31</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>9462.559999999999</v>
+        <v>9516.6</v>
       </c>
     </row>
     <row r="13">
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>9462.559999999999</v>
+        <v>9516.6</v>
       </c>
     </row>
     <row r="14">
@@ -636,7 +636,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>-1419.38</v>
+        <v>-1427.49</v>
       </c>
     </row>
     <row r="15">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>8043.18</v>
+        <v>8089.11</v>
       </c>
     </row>
     <row r="16">
@@ -680,23 +680,13 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Cash Payments Owed</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>-224</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Net to Doral</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n">
-        <v>7086.82</v>
+      <c r="B19" s="6" t="n">
+        <v>7356.75</v>
       </c>
     </row>
   </sheetData>
@@ -8733,7 +8723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -8818,106 +8808,99 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2. Ocean Harbor Ertas Meral (+$118.91) and Morin George (−$64.87) are on Doral's Pearl statement (producer 6883)</t>
+          <t>2. Ocean Harbor is recorded in full as its producer-6883 statement shows: all five lines including Ertas Meral</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   but their policy numbers are not in the binder book, so by the policy-number rule they are excluded (net</t>
+          <t xml:space="preserve">   (+$118.91) and Morin George (−$64.87), so the section foots to the statement's $250.08 Commission Due.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   +$54.04). Include them if producer code 6883 is Doral-exclusive.</t>
+          <t>3. Office-only expense lines are 220 License Rent ($500) and Systems ($224), provided for July; the Cash Payments</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3. Office-only expense lines (220 License Rent, Systems, Cash Payments Owed) carry June's figures forward as</t>
+          <t xml:space="preserve">   Owed line has been removed for now. They appear on no carrier statement.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   placeholders — they appear on no carrier statement. Confirm the July amounts.</t>
-        </is>
-      </c>
+      <c r="A17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>BINDER POLICIES WITH NO CARRIER COMMISSION THIS MONTH ($0 — likely billed in an adjacent statement period):</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>BINDER POLICIES WITH NO CARRIER COMMISSION THIS MONTH ($0 — likely billed in an adjacent statement period):</t>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    LUIS CHACON PENA  |  Progressive  |  Renewed  |  991253124</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">    LUIS CHACON PENA  |  Progressive  |  Renewed  |  991253124</t>
+          <t xml:space="preserve">    EMILEY BLOMBERG  |  Progressive  |  Renewed  |  999745921</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">    EMILEY BLOMBERG  |  Progressive  |  Renewed  |  999745921</t>
+          <t xml:space="preserve">    GUILLERMO FAYAS RODRIGUEZ  |  Progressive  |  Renewed  |  867943703</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">    GUILLERMO FAYAS RODRIGUEZ  |  Progressive  |  Renewed  |  867943703</t>
+          <t xml:space="preserve">    KAREN A MORALES  |  Progressive  |  Pending  |  971858902</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">    KAREN A MORALES  |  Progressive  |  Pending  |  971858902</t>
+          <t xml:space="preserve">    HECTOR L PARRA SALCEDO  |  Progressive  |  Active  |  973393972</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    HECTOR L PARRA SALCEDO  |  Progressive  |  Active  |  973393972</t>
+          <t xml:space="preserve">    ALEX CRUZ  |  Ocean Harbor  |  Active  |  P020072668104</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ALEX CRUZ  |  Ocean Harbor  |  Active  |  P020072668104</t>
+          <t xml:space="preserve">    TAMMIE GOA  |  Ocean Harbor  |  Active  |  P020073692004</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    TAMMIE GOA  |  Ocean Harbor  |  Active  |  P020073692004</t>
+          <t xml:space="preserve">    KEVIN D. JIMENEZ AGUERO  |  National General  |  Active  |  2033211242</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    KEVIN D. JIMENEZ AGUERO  |  National General  |  Active  |  2033211242</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
         <is>
           <t xml:space="preserve">    ALBA VASQUEZ  |  Infinity  |  Renewed  |  10214575901</t>
         </is>

</xml_diff>